<commit_message>
Update Excel for form
</commit_message>
<xml_diff>
--- a/assets/floor_2_data.xlsx
+++ b/assets/floor_2_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M.Mead\9.FactoryView\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB780C76-8EFD-43AC-8C9D-9F056736C520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94138BE5-3657-4AA8-96E8-166F2D8326CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loc_name" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,13 @@
     <sheet name="prod_comp" sheetId="9" r:id="rId3"/>
     <sheet name="machine" sheetId="8" r:id="rId4"/>
     <sheet name="form_can_1" sheetId="12" r:id="rId5"/>
-    <sheet name="weight" sheetId="6" r:id="rId6"/>
-    <sheet name="zones" sheetId="5" r:id="rId7"/>
-    <sheet name="zones_noname" sheetId="13" r:id="rId8"/>
-    <sheet name="flow_powder" sheetId="11" r:id="rId9"/>
-    <sheet name="flow_pouch" sheetId="7" r:id="rId10"/>
-    <sheet name="flow_can" sheetId="10" r:id="rId11"/>
+    <sheet name="form_pouch_1" sheetId="14" r:id="rId6"/>
+    <sheet name="weight" sheetId="6" r:id="rId7"/>
+    <sheet name="zones" sheetId="5" r:id="rId8"/>
+    <sheet name="zones_noname" sheetId="13" r:id="rId9"/>
+    <sheet name="flow_powder" sheetId="11" r:id="rId10"/>
+    <sheet name="flow_pouch" sheetId="7" r:id="rId11"/>
+    <sheet name="flow_can" sheetId="10" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -87,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="295">
   <si>
     <t>Name</t>
   </si>
@@ -878,9 +879,6 @@
     <t>assets/docs/1000391098+5000006870_CAN/5.Blender/Process_P_011.pdf</t>
   </si>
   <si>
-    <t>Tipping Record - Operator</t>
-  </si>
-  <si>
     <t>assets/docs/1000391098+5000006870_CAN/5.Blender/Process_P_112.pdf</t>
   </si>
   <si>
@@ -936,6 +934,45 @@
   </si>
   <si>
     <t>#fcbe03</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/4.Dispensing/Process_P_108.pdf</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/5.Blender/Process_P_097.pdf</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/5.Blender/Process_P_119.pdf</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/5.Blender/Process_P_013.pdf</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/5.Blender/Process_P_095.pdf</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/5.Blender/Machine_P_043_044.pdf</t>
+  </si>
+  <si>
+    <t>Tipping Record (CCP1)</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/6.Vitamin%20Weighing/Machine_P_103.pdf</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/6.Vitamin%20Weighing/Machine_P_104.pdf</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/6.Vitamin%20Weighing/Process_P_101.pdf</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/6.Vitamin%20Weighing/Process_P_102.pdf</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/7.Sifter/Machine_P_006_007.pdf</t>
+  </si>
+  <si>
+    <t>assets/docs/1000381996+1000381979_POUCH/7.Sifter/Machine_P_045.pdf</t>
   </si>
 </sst>
 </file>
@@ -1038,7 +1075,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1068,6 +1105,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1489,6 +1527,332 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57EE0D85-DD60-4891-B20F-895CEC338B14}">
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.21875" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="112" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.44140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="7.21875" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.88671875" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="D2" s="10">
+        <v>2</v>
+      </c>
+      <c r="E2" s="10">
+        <v>30</v>
+      </c>
+      <c r="F2" s="10">
+        <v>15</v>
+      </c>
+      <c r="G2" s="10">
+        <v>0</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="I2" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" s="10">
+        <v>2</v>
+      </c>
+      <c r="E3" s="10">
+        <v>30</v>
+      </c>
+      <c r="F3" s="10">
+        <v>15</v>
+      </c>
+      <c r="G3" s="10">
+        <v>0</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="I3" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="D4" s="10">
+        <v>2</v>
+      </c>
+      <c r="E4" s="10">
+        <v>30</v>
+      </c>
+      <c r="F4" s="10">
+        <v>15</v>
+      </c>
+      <c r="G4" s="10">
+        <v>0</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="I4" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" s="10">
+        <v>2</v>
+      </c>
+      <c r="E5" s="10">
+        <v>30</v>
+      </c>
+      <c r="F5" s="10">
+        <v>15</v>
+      </c>
+      <c r="G5" s="10">
+        <v>0</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="I5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="D6" s="10">
+        <v>1</v>
+      </c>
+      <c r="E6" s="10">
+        <v>20</v>
+      </c>
+      <c r="F6" s="10">
+        <v>5</v>
+      </c>
+      <c r="G6" s="10">
+        <v>0</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="I6" s="10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="D7" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="E7" s="10">
+        <v>20</v>
+      </c>
+      <c r="F7" s="10">
+        <v>5</v>
+      </c>
+      <c r="G7" s="10">
+        <v>0.2</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="I7" s="10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="D8" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="10">
+        <v>20</v>
+      </c>
+      <c r="F8" s="10">
+        <v>5</v>
+      </c>
+      <c r="G8" s="10">
+        <v>0.2</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="I8" s="10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="D9" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="E9" s="10">
+        <v>20</v>
+      </c>
+      <c r="F9" s="10">
+        <v>5</v>
+      </c>
+      <c r="G9" s="10">
+        <v>0.2</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="I9" s="10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="D10" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="10">
+        <v>20</v>
+      </c>
+      <c r="F10" s="10">
+        <v>5</v>
+      </c>
+      <c r="G10" s="10">
+        <v>0.2</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="I10" s="10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4FA26C3-CAFB-4728-933F-28CE0AA88343}">
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1687,7 +2051,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AC33B8A-E190-477F-A359-A40597F7270D}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3206,7 +3570,7 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="12" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>0</v>
@@ -3215,7 +3579,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E1" s="10" t="s">
         <v>2</v>
@@ -3265,7 +3629,7 @@
         <v>235</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E2" s="11">
         <v>626</v>
@@ -3294,7 +3658,7 @@
         <v>235</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E3" s="11">
         <v>780</v>
@@ -3317,13 +3681,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E4" s="11">
         <v>780</v>
@@ -3361,7 +3725,7 @@
         <v>235</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E5" s="11">
         <v>780</v>
@@ -3376,7 +3740,7 @@
         <v>240</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -3384,13 +3748,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>263</v>
+        <v>288</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E6" s="11">
         <v>780</v>
@@ -3402,10 +3766,10 @@
         <v>239</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -3413,25 +3777,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E7" s="11">
         <v>1240</v>
       </c>
       <c r="F7" s="11">
-        <v>-574</v>
+        <v>-570</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>243</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K7" s="11" t="s">
         <v>244</v>
@@ -3439,176 +3803,176 @@
     </row>
     <row r="8" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="13">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>281</v>
-      </c>
-      <c r="E8" s="11">
+        <v>280</v>
+      </c>
+      <c r="E8" s="17">
         <v>892</v>
       </c>
       <c r="F8" s="11">
         <v>-855</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="13">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>281</v>
-      </c>
-      <c r="E9" s="11">
+        <v>280</v>
+      </c>
+      <c r="E9" s="17">
         <v>1126</v>
       </c>
       <c r="F9" s="11">
         <v>-855</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J9" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="13">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>281</v>
-      </c>
-      <c r="E10" s="11">
+        <v>280</v>
+      </c>
+      <c r="E10" s="17">
         <v>1291</v>
       </c>
       <c r="F10" s="11">
         <v>-855</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="13">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>281</v>
-      </c>
-      <c r="E11" s="11">
+        <v>280</v>
+      </c>
+      <c r="E11" s="17">
         <v>892</v>
       </c>
       <c r="F11" s="11">
         <v>-820</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J11" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="13">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>281</v>
-      </c>
-      <c r="E12" s="11">
+        <v>280</v>
+      </c>
+      <c r="E12" s="17">
         <v>1126</v>
       </c>
       <c r="F12" s="11">
         <v>-820</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>281</v>
-      </c>
-      <c r="E13" s="11">
+        <v>280</v>
+      </c>
+      <c r="E13" s="17">
         <v>1291</v>
       </c>
       <c r="F13" s="11">
         <v>-820</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -3616,13 +3980,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E14" s="11">
         <v>1210</v>
@@ -3631,13 +3995,13 @@
         <v>-190</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="16" customFormat="1" x14ac:dyDescent="0.2">
@@ -3645,13 +4009,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>235</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E15" s="16">
         <v>1210</v>
@@ -3660,13 +4024,13 @@
         <v>-160</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="J15" s="16" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K15" s="16" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="16" customFormat="1" x14ac:dyDescent="0.2">
@@ -3674,13 +4038,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>235</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E16" s="16">
         <v>1210</v>
@@ -3689,13 +4053,13 @@
         <v>-130</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="J16" s="16" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="K16" s="16" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -3706,6 +4070,443 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FB71D57-BE2D-4E53-8949-88C80A2C6281}">
+  <dimension ref="A1:P13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="12"/>
+    <col min="2" max="2" width="38.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" style="10" customWidth="1"/>
+    <col min="5" max="5" width="5" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.21875" style="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76" style="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.21875" style="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9" style="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="50.21875" style="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="63.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="8.88671875" style="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="N1" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="O1" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="P1" s="10" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="13">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="E2" s="11">
+        <v>626</v>
+      </c>
+      <c r="F2" s="11">
+        <v>-950</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="13">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="E3" s="11">
+        <v>950</v>
+      </c>
+      <c r="F3" s="11">
+        <v>-630</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="13">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="E4" s="11">
+        <v>950</v>
+      </c>
+      <c r="F4" s="11">
+        <v>-600</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="M4" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="N4" s="11" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="13">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="E5" s="11">
+        <v>950</v>
+      </c>
+      <c r="F5" s="11">
+        <v>-570</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="13">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="E6" s="11">
+        <v>950</v>
+      </c>
+      <c r="F6" s="11">
+        <v>-540</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>281</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="13">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="E7" s="11">
+        <v>1240</v>
+      </c>
+      <c r="F7" s="11">
+        <v>-540</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="13">
+        <v>8</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="E8" s="11">
+        <v>1291</v>
+      </c>
+      <c r="F8" s="11">
+        <v>-855</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="13">
+        <v>9</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="E9" s="11">
+        <v>892</v>
+      </c>
+      <c r="F9" s="11">
+        <v>-855</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="13">
+        <v>11</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="E10" s="11">
+        <v>1291</v>
+      </c>
+      <c r="F10" s="11">
+        <v>-820</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="J10" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="13">
+        <v>12</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="E11" s="11">
+        <v>892</v>
+      </c>
+      <c r="F11" s="11">
+        <v>-820</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="J11" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="13">
+        <v>13</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="E12" s="11">
+        <v>1330</v>
+      </c>
+      <c r="F12" s="11">
+        <v>-430</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>268</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="16" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="15">
+        <v>14</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>273</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="E13" s="16">
+        <v>1330</v>
+      </c>
+      <c r="F13" s="16">
+        <v>-400</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="J13" s="16" t="s">
+        <v>281</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>294</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A113FB90-F9A2-4A63-A07C-A429C0E9DE7B}">
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3886,7 +4687,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4333,7 +5134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BE13484-8EF2-4DFC-A1DA-64C2CD377CCC}">
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4747,330 +5548,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57EE0D85-DD60-4891-B20F-895CEC338B14}">
-  <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="16.21875" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="112" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.44140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.77734375" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="7.21875" style="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.88671875" style="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.5546875" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="J1" s="10" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="D2" s="10">
-        <v>2</v>
-      </c>
-      <c r="E2" s="10">
-        <v>30</v>
-      </c>
-      <c r="F2" s="10">
-        <v>15</v>
-      </c>
-      <c r="G2" s="10">
-        <v>0</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="I2" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="J2" s="10" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="D3" s="10">
-        <v>2</v>
-      </c>
-      <c r="E3" s="10">
-        <v>30</v>
-      </c>
-      <c r="F3" s="10">
-        <v>15</v>
-      </c>
-      <c r="G3" s="10">
-        <v>0</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="I3" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="D4" s="10">
-        <v>2</v>
-      </c>
-      <c r="E4" s="10">
-        <v>30</v>
-      </c>
-      <c r="F4" s="10">
-        <v>15</v>
-      </c>
-      <c r="G4" s="10">
-        <v>0</v>
-      </c>
-      <c r="H4" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="I4" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="D5" s="10">
-        <v>2</v>
-      </c>
-      <c r="E5" s="10">
-        <v>30</v>
-      </c>
-      <c r="F5" s="10">
-        <v>15</v>
-      </c>
-      <c r="G5" s="10">
-        <v>0</v>
-      </c>
-      <c r="H5" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="I5" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="D6" s="10">
-        <v>1</v>
-      </c>
-      <c r="E6" s="10">
-        <v>20</v>
-      </c>
-      <c r="F6" s="10">
-        <v>5</v>
-      </c>
-      <c r="G6" s="10">
-        <v>0</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="I6" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="D7" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="E7" s="10">
-        <v>20</v>
-      </c>
-      <c r="F7" s="10">
-        <v>5</v>
-      </c>
-      <c r="G7" s="10">
-        <v>0.2</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="I7" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="D8" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="E8" s="10">
-        <v>20</v>
-      </c>
-      <c r="F8" s="10">
-        <v>5</v>
-      </c>
-      <c r="G8" s="10">
-        <v>0.2</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="I8" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="D9" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="E9" s="10">
-        <v>20</v>
-      </c>
-      <c r="F9" s="10">
-        <v>5</v>
-      </c>
-      <c r="G9" s="10">
-        <v>0.2</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="I9" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>210</v>
-      </c>
-      <c r="D10" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="E10" s="10">
-        <v>20</v>
-      </c>
-      <c r="F10" s="10">
-        <v>5</v>
-      </c>
-      <c r="G10" s="10">
-        <v>0.2</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="I10" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>